<commit_message>
Move canonical food log xlsx into repo data/.
</commit_message>
<xml_diff>
--- a/data/fitness_food_log.xlsx
+++ b/data/fitness_food_log.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="48" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
           <t>2026-09-05</t>
@@ -2658,40 +2658,803 @@
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="inlineStr">
+        <is>
+          <t>Fete Up lunch（用戶約 490）</t>
+        </is>
+      </c>
+      <c r="D105" s="1" t="n">
+        <v>490</v>
+      </c>
+      <c r="E105" s="1" t="n">
+        <v>430</v>
+      </c>
+      <c r="F105" s="1" t="n">
+        <v>560</v>
+      </c>
+      <c r="G105" s="1" t="inlineStr">
+        <is>
+          <t>已食。跟她報 Record 490。未報分項／碟相，未拆。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="84" customHeight="1">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="C105" s="1" t="inlineStr">
-        <is>
-          <t>預估：Feather &amp; Bone CWB RW 2人套餐；T-bone 1kg share 50%；頭盤50%；前菜暫按他他；甜品暫按芝士蛋糕；wine 220mL</t>
-        </is>
-      </c>
-      <c r="D105" s="1" t="n">
-        <v>2320</v>
-      </c>
-      <c r="E105" s="1" t="n">
-        <v>1950</v>
-      </c>
-      <c r="F105" s="1" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G105" s="1" t="inlineStr">
-        <is>
-          <t>未食。假設2人分1kg T-bone。DiningCity食客實拍：T-bone連薯～1580全份／半份790；頭盤～1100／半份550；他他＋crostini～395；FAB芝士蛋糕暫400（未有清晰碟相）；wine220mL×83＝183。合計2320。若松露通心粉球＋朱古力蛋糕可去～2700。Gallery薯條唔自動加入RW T-bone（食客相無薯條）。有實點改同一行。</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="C106" s="1" t="n"/>
-    </row>
-    <row r="107">
-      <c r="C107" s="1" t="n"/>
+      <c r="C106" s="1" t="inlineStr">
+        <is>
+          <t>F&amp;B CWB RW：頭盤前菜＋甜品50/50；T-bone 你約4塊；薯條≤10；wine 約300mL</t>
+        </is>
+      </c>
+      <c r="D106" s="1" t="n">
+        <v>2590</v>
+      </c>
+      <c r="E106" s="1" t="n">
+        <v>2390</v>
+      </c>
+      <c r="F106" s="1" t="n">
+        <v>2840</v>
+      </c>
+      <c r="G106" s="1" t="inlineStr">
+        <is>
+          <t>同一行改：酒由暫400mL改用戶約300mL×83＝249（先前330）。牛扒4塊＝520、頭盤前菜960、甜品640、薯條220不變。合計2590。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="48" customHeight="1">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch Fete Up＋F&amp;B dinner含酒）</t>
+        </is>
+      </c>
+      <c r="D107" s="1" t="n">
+        <v>3080</v>
+      </c>
+      <c r="E107" s="1" t="n">
+        <v>2820</v>
+      </c>
+      <c r="F107" s="1" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G107" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch490＋dinner2590＝3080。同一行由3160改（酒約300mL）。未報早餐／其他＝未計。空白≠0。</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="C108" s="1" t="n"/>
-    </row>
-    <row r="109">
-      <c r="C109" s="1" t="n"/>
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="inlineStr">
+        <is>
+          <t>枝豆少量（未秤）</t>
+        </is>
+      </c>
+      <c r="D108" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E108" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F108" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G108" s="1" t="inlineStr">
+        <is>
+          <t>未秤。按連殼約40g×53%出肉＝21g豆×121kcal/100g＝26，記30。蛋白約4g。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="48" customHeight="1">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>已食：烚蝦5中大隻＋蒸魚肉200g清蒸＋水蛋一些＋菜心一些＋火龍果大2個÷3</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="n">
+        <v>580</v>
+      </c>
+      <c r="E109" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="F109" s="1" t="n">
+        <v>700</v>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t>已食，同一行改預估。蝦5中大隻按可食約110g×99＝110。魚肉200g清蒸×110＝220。水蛋一些按約1隻蛋多啲＝90。菜心一些無油＝30。火龍果大2÷3：每個可食約340g×50kcal/100g＝170，2個＝340÷3＝113，記130。合計580。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="36" customHeight="1">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C110" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 枝豆＋dinner 蒸魚蝦水蛋菜心火龍果）</t>
+        </is>
+      </c>
+      <c r="D110" s="1" t="n">
+        <v>610</v>
+      </c>
+      <c r="E110" s="1" t="n">
+        <v>520</v>
+      </c>
+      <c r="F110" s="1" t="n">
+        <v>750</v>
+      </c>
+      <c r="G110" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch30＋dinner580＝610。偏低；空白≠0。未報早餐／其他＝未計。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C111" s="1" t="inlineStr">
+        <is>
+          <t>蛋2隻＋沙律菜60g無醬</t>
+        </is>
+      </c>
+      <c r="D111" s="1" t="n">
+        <v>165</v>
+      </c>
+      <c r="E111" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F111" s="1" t="n">
+        <v>220</v>
+      </c>
+      <c r="G111" s="1" t="inlineStr">
+        <is>
+          <t>已食。蛋2隻未講煮法，按無油＝150。沙律60g無醬＝15。合計165。有油改同一行。蛋白約12g。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C112" s="1" t="inlineStr">
+        <is>
+          <t>已併入晚餐（枝豆）</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="n"/>
+      <c r="E112" s="1" t="n"/>
+      <c r="F112" s="1" t="n"/>
+      <c r="G112" s="1" t="inlineStr">
+        <is>
+          <t>同一日枝豆改入 Dinner 行，避免重複。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="60" customHeight="1">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C113" s="1" t="inlineStr">
+        <is>
+          <t>晚餐：烚蝦4隻連殼125g＋生菜大量＋枝豆連殼125g＋水果一半（蘋1個＋紅火龍果約180g 全碟，食一半）</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="n">
+        <v>290</v>
+      </c>
+      <c r="E113" s="1" t="n">
+        <v>240</v>
+      </c>
+      <c r="F113" s="1" t="n">
+        <v>360</v>
+      </c>
+      <c r="G113" s="1" t="inlineStr">
+        <is>
+          <t>已食。同一行加枝豆＋水果。蝦連殼125g出肉79g＝80。生菜大量無醬＝30。枝豆連殼125g×53%＝66g豆＝80。水果全碟蘋約90＋火龍果約110＝200，食一半＝100。合計290。吸頭已包在出肉。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 蛋沙律＋dinner 蝦生菜枝豆水果一半）</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="n">
+        <v>455</v>
+      </c>
+      <c r="E114" s="1" t="n">
+        <v>390</v>
+      </c>
+      <c r="F114" s="1" t="n">
+        <v>580</v>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch165＋dinner290＝455。偏低；空白≠0。未報早餐／其他＝未計。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="36" customHeight="1">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C115" s="1" t="inlineStr">
+        <is>
+          <t>蛋2隻＋沙律菜60g無醬</t>
+        </is>
+      </c>
+      <c r="D115" s="1" t="n">
+        <v>165</v>
+      </c>
+      <c r="E115" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F115" s="1" t="n">
+        <v>220</v>
+      </c>
+      <c r="G115" s="1" t="inlineStr">
+        <is>
+          <t>已食。蛋2隻未講煮法，按無油＝150。沙律60g無醬＝15。合計165。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="72" customHeight="1">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C116" s="1" t="inlineStr">
+        <is>
+          <t>家上海：雲吞雞她份（雲吞4＋雞¼去皮＋菜＋湯約5小碗）＋乳鴿去皮¼＋小籠包3隻</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="n">
+        <v>1190</v>
+      </c>
+      <c r="E116" s="1" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F116" s="1" t="n">
+        <v>1360</v>
+      </c>
+      <c r="G116" s="1" t="inlineStr">
+        <is>
+          <t>已食＋碟相＋去皮。同一行。小籠3＝276。雲吞4＝400。雞¼去皮熟肉約115g＝190（連皮300改）。菜20。湯5小碗約850mL＝240。乳鴿去皮¼＝70。合計1196記1190。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="36" customHeight="1">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C117" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 蛋沙律＋dinner 家上海）</t>
+        </is>
+      </c>
+      <c r="D117" s="1" t="n">
+        <v>1355</v>
+      </c>
+      <c r="E117" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F117" s="1" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G117" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch165＋dinner1190＝1355。未報早餐／其他＝未計。空白≠0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C118" s="1" t="inlineStr">
+        <is>
+          <t>沙律菜＋牛肉</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="E118" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="F118" s="1" t="n">
+        <v>180</v>
+      </c>
+      <c r="G118" s="1" t="inlineStr">
+        <is>
+          <t>已食。用戶報沙律菜＋牛肉＝150。跟她報嘅數。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="48" customHeight="1">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>大量菜＋yoghurt 170g＋雞柳約65g＋果泥約50＋蘋果2個÷3</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="n">
+        <v>335</v>
+      </c>
+      <c r="E119" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F119" s="1" t="n">
+        <v>420</v>
+      </c>
+      <c r="G119" s="1" t="inlineStr">
+        <is>
+          <t>已食。同一行加蘋果：2個中個約94×2＝188，3人share她⅓＝63記65。yoghurt104＋雞柳78＋果泥50＋菜40＋蘋果65＝335。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="36" customHeight="1">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 沙律牛肉＋dinner 菜yoghurt雞柳果泥蘋果）</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="n">
+        <v>485</v>
+      </c>
+      <c r="E120" s="1" t="n">
+        <v>410</v>
+      </c>
+      <c r="F120" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch150＋dinner335＝485。偏低；空白≠0。未報早餐／其他＝未計。唔當還二1,355。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="56" customHeight="1">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>蒟蒻麵＋雞柳＋蝦＋青口＋枝豆（相未見枝豆）</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="n">
+        <v>260</v>
+      </c>
+      <c r="E121" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="F121" s="1" t="n">
+        <v>330</v>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>已食。9/11 00:24報，當9/10 lunch。蒟蒻20＋雞柳65＋蝦35＋青口55＋蘿蔔20＋湯油25＋枝豆暫40。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C122" s="1" t="inlineStr">
+        <is>
+          <t>下午茶：韓國香印提子約130g</t>
+        </is>
+      </c>
+      <c r="D122" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="E122" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="F122" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="G122" s="1" t="inlineStr">
+        <is>
+          <t>已食。130g x0.70=91記90。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="48" customHeight="1">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C123" s="1" t="inlineStr">
+        <is>
+          <t>烚蝦2＋青口6–7＋鰹魚粉蛋花紫菜湯＋菜心大量</t>
+        </is>
+      </c>
+      <c r="D123" s="1" t="n">
+        <v>340</v>
+      </c>
+      <c r="E123" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F123" s="1" t="n">
+        <v>420</v>
+      </c>
+      <c r="G123" s="1" t="inlineStr">
+        <is>
+          <t>已食。蝦40＋青口140＋鰹魚粉20＋蛋75＋紫菜10＋菜心40＋湯汁15=340。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="36" customHeight="1">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C124" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 蒟蒻碗＋下午茶香印＋dinner 蝦青口蛋花湯）</t>
+        </is>
+      </c>
+      <c r="D124" s="1" t="n">
+        <v>690</v>
+      </c>
+      <c r="E124" s="1" t="n">
+        <v>560</v>
+      </c>
+      <c r="F124" s="1" t="n">
+        <v>850</v>
+      </c>
+      <c r="G124" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch260＋香印90＋dinner340=690。偏低；空白≠0。未報早餐／其他＝未計。唔當還。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="72" customHeight="1">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>清蒸魚一條420g（連頭骨假設）食2/3＋醬油＋蝦5隻＋生菜大量。魚：可食約50%→210g，2/3≈140g熟肉×115＝161＋醬油你份20＝181。蝦5未秤，按中隻可食約100g白灼×99＝99。生菜大量無醬＝30（同9/7）。淋咗熱油再改同一行。</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="n">
+        <v>310</v>
+      </c>
+      <c r="E125" s="1" t="n">
+        <v>220</v>
+      </c>
+      <c r="F125" s="1" t="n">
+        <v>400</v>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>已食。420g當連頭骨一條，可食率假設50%（未秤骨）。魚種未報，按白肉清蒸115kcal/100g。蝦未報煮法／連殼重，當白灼無油。生菜未秤、無醬。未日結。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="88" customHeight="1">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B126" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C126" s="1" t="inlineStr">
+        <is>
+          <t>已食：米紙卷4.5＋雞柳65g生＋吞拿魚50＋雞肉鬆40＋yoghurt醬50＋菜20＋鯖魚柳60g生＝490。枝豆100g連殼65＋ham 3片70（維持）。啤酒530mL×29kcal/100mL＝154（取代舊200）。紅酒100mL×83＝83。另＋100 buffer（你報）。490＋65＋70＋154＋83＋100＝962，記960。</t>
+        </is>
+      </c>
+      <c r="D126" s="1" t="n">
+        <v>960</v>
+      </c>
+      <c r="E126" s="1" t="n">
+        <v>900</v>
+      </c>
+      <c r="F126" s="1" t="n">
+        <v>1060</v>
+      </c>
+      <c r="G126" s="1" t="inlineStr">
+        <is>
+          <t>同一行。啤酒改實數530mL×29/100mL＝154；紅酒100mL＝83；枝豆／ham維持65／70當已食；＋100 buffer。舊未食335*同舊啤酒200刪。已食。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="48" customHeight="1">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B127" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C127" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 310＋dinner 960）</t>
+        </is>
+      </c>
+      <c r="D127" s="1" t="n">
+        <v>1270</v>
+      </c>
+      <c r="E127" s="1" t="n">
+        <v>1120</v>
+      </c>
+      <c r="F127" s="1" t="n">
+        <v>1460</v>
+      </c>
+      <c r="G127" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch 310＋dinner 960＝1,270。未報早餐＝未計。空白≠0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="56" customHeight="1">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B128" s="1" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C128" s="1" t="inlineStr">
+        <is>
+          <t>蝦約6隻中小型＋墨魚滑約70g＋提子1粒。蝦可食約90g×99＝89；墨魚滑70×120＝84；提子1粒≈10。89＋84＋10＝183，記185。</t>
+        </is>
+      </c>
+      <c r="D128" s="1" t="n">
+        <v>185</v>
+      </c>
+      <c r="E128" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F128" s="1" t="n">
+        <v>240</v>
+      </c>
+      <c r="G128" s="1" t="inlineStr">
+        <is>
+          <t>同一行加提子1粒≈10（晴王級約10；普通提子約6–8）。蝦／墨魚滑假設不變。有油再改。未日結。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="96" customHeight="1">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B129" s="1" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C129" s="1" t="inlineStr">
+        <is>
+          <t>已食相＋你更正。前菜÷6＝359。魚半手大＋煎皮130；牛三四口130；鴨幾口60。烤薯＋烤蘿蔔食咗D＝120。甜品÷6＝333。額外麵包你自己：相係咬一口後，當全片約80g＝200＋一些牛油50＝250（舊80刪）。酒0。359＋130＋130＋60＋120＋333＋250＝1,382，記1,380。</t>
+        </is>
+      </c>
+      <c r="D129" s="1" t="n">
+        <v>1380</v>
+      </c>
+      <c r="E129" s="1" t="n">
+        <v>1090</v>
+      </c>
+      <c r="F129" s="1" t="n">
+        <v>1790</v>
+      </c>
+      <c r="G129" s="1" t="inlineStr">
+        <is>
+          <t>同一行。額外麵包改：一口後拍照＝其餘都食；有牛油。由80改250。酒0。日結見 Total。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B130" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C130" s="1" t="inlineStr">
+        <is>
+          <t>日結（lunch 185＋dinner 1,380）</t>
+        </is>
+      </c>
+      <c r="D130" s="1" t="n">
+        <v>1565</v>
+      </c>
+      <c r="E130" s="1" t="n">
+        <v>1240</v>
+      </c>
+      <c r="F130" s="1" t="n">
+        <v>2030</v>
+      </c>
+      <c r="G130" s="1" t="inlineStr">
+        <is>
+          <t>日結。lunch 185＋dinner 1,380＝1,565。酒0。未報早餐＝未計。空白≠0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" s="1" t="n"/>
+    </row>
+    <row r="132">
+      <c r="C132" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G4"/>
@@ -2900,8 +3663,12 @@
       <c r="G4" s="6" t="n">
         <v>3745</v>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>3080</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>610</v>
+      </c>
       <c r="J4" s="6">
         <f>COUNTA(C4:I4)</f>
         <v/>
@@ -2916,7 +3683,7 @@
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>一470日結（偏低）；二735日結（偏低，gym日）；三1010日結；四666日結；五3745日結（Nissa RW＋wine5＋cocktail抹茶蓋）。其餘空白≠0。週合計／平均用COUNTA只計有記日。</t>
+          <t>一470；二735；三1010；四666；五3745（Nissa）；六3080（F&amp;B）；日610日結（偏低）。週合計10316，平均1474。超9800約516。空白≠0。</t>
         </is>
       </c>
     </row>
@@ -2927,12 +3694,24 @@
       <c r="B5" s="10" t="n">
         <v>46278</v>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
+      <c r="C5" s="6" t="n">
+        <v>455</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1355</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>485</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>690</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>1270</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>1565</v>
+      </c>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6">
         <f>COUNTA(C5:I5)</f>
@@ -2946,7 +3725,11 @@
         <f>IF(J5=0,"",ROUND(K5/J5,0))</f>
         <v/>
       </c>
-      <c r="M5" s="8" t="n"/>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>一455；二1355；三485；四690；五1270；六1565日結。日空白≠0。有記6日合計5,820，平均970。偏低日唔當還。</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="10" t="n">
@@ -3056,7 +3839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3558,6 +4341,226 @@
       <c r="E26" s="1" t="inlineStr">
         <is>
           <t>完成。重量7機。Chest 15太重停7.5；pulldown 冇12kg停10；glute 4×10@12。腿抖 skip 機上行。用戶行700m回家當 walk。無錶數據，唔估kcal、唔扣食物。聽日（五）腿休息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 morning</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 63.5。用戶更正日期：係9/5晨，唔係9/6。較9/4晨 63.5 持平。尋晚 Nissa 3,745 嘅鈉／酒水可能當日稍後或9/6先上秤，唔當減脂、唔當新底。7日晨磅均約63.5（8/30–9/5：63.75／64.25／63.2／63.0／63.3／63.5／63.5）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 morning</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="C28" s="1" t="n"/>
+      <c r="D28" s="1" t="n"/>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 63.9（下午報）。較9/5晨 63.5 ＋0.4。尋晚 F&amp;B 鈉／酒／肝醣／腸胃內容物，唔當增脂、唔當新底。7日晨磅均約63.5（8/31–9/6：64.25／63.2／63.0／63.3／63.5／63.5／63.9）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 gym（完成）</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>Hip abduction 5×12 @25kg；Hip adduction 4×12 @15kg；Squat machine 3×10 @2.5kg；Chest press 5×10 @7.5kg；Glute drive 3×12 @12.5kg</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>Star Trac Indoor Run 17:43-18:27；44:25；2.90km；爬升253m；pace 15'19"/km；avg HR127（peak約142）；cadence71；Effort4 Moderate；active184／total247 kcal（手錶，唔扣食物）。Splits：15:19 HR124；15:00 HR127；14:01 HR130。</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>完成。重量：hip ab 5×12@25（向外推）；hip ad 4×12@15（齊12）；squat 3×10@2.5；chest 5×10@7.5；glute 3×12@12.5。Cardio：Star Trac 44:25／2.90km／爬升253m（約8.7%），HR127 Moderate。計劃40分斜7%；實際多分4分、斜略高。手錶184／247唔扣食物。聽日腿休息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 morning</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="C30" s="1" t="n"/>
+      <c r="D30" s="1" t="n"/>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 63.5。較9/6晨 63.9 −0.4。尋晚 F&amp;B 水回落，唔當一日減脂、唔當新底。7日晨磅均約63.4（9/1–9/7：63.2／63.0／63.3／63.5／63.5／63.9／63.5）。今日腿休息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 morning</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>62.65</v>
+      </c>
+      <c r="C31" s="1" t="n"/>
+      <c r="D31" s="1" t="n"/>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 62.65。較9/7晨 63.5 −0.85。尋日全日455偏低＋F&amp;B水繼續走，腸空／肝醣水，唔當減脂、唔當新底。7日晨磅均約63.3（9/2–9/8：63.0／63.3／63.5／63.5／63.9／63.5／62.65）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 morning</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>62.95</v>
+      </c>
+      <c r="C32" s="1" t="n"/>
+      <c r="D32" s="1" t="n"/>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 62.95。較9/8晨 62.65 ＋0.30。尋日日結1355後回水／腸胃，唔當增脂、唔當新底。9/8嘅62.65係455後日腸空，唔係 dry。7日晨磅均仍約63.3（9/3–9/9：63.3／63.5／63.5／63.9／63.5／62.65／62.95）。 今日（三）唔得閒 gym，改四開始。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 gym（完成）</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>Hip Abduction 4x10 @30kg; Hip Adduction 4x10 @15kg; Leg Press 4x10 @15kg; Wide Pulldown 4x8 @15kg; Chest Press 4x12 @7.5kg; Pectoral Fly 4x10 @10kg; Squat Machine 4x10 @2.5kg</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>Star Trac Indoor Run 18:14-18:57; 43:14; 2.66km; climb 229m; pace 16'17"/km; avg HR132; cadence82; Effort4 Moderate; active152 / total212 kcal (watch, never subtract from food). Splits: 16:21 HR121; 16:34 HR141; 10:19 HR134.</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Done. Weights as table. App volume 3740 kg. Cardio 43:14 / 2.66km / climb 229m (~8.6%), HR132 Moderate. Watch 152/212 not subtracted. Pec fly = chest not back. Extra LP/fly logged as-is; do not add more machines next time. Fri: no extra cardio (already 43 min incline Thu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 afternoon home</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="n"/>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>晏晝在家秤 62.55。唔當晨磅。較今晨未報；較 9/9 晨 62.95 −0.40，條件唔同（下午／gym 前），當水／腸胃，唔當新底／減脂。7 日晨磅均仍用晨間。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="88" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:56 gym BIA</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="C35" s="1" t="n"/>
+      <c r="D35" s="1" t="n"/>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>HowBodyFit 2026-09-10 17:56（女30／160cm，gym room，Star Trac 前）：Score69；體重62.7；BMI24.5 normal；BFP35.1% High；BMR1249；代謝年齡35。水29.6、蛋白8.1、礦物質3.0、ICF18.5、ECF11.1 均 normal。骨骼肌22.1、去脂40.7 normal；體脂22.0 High。WHR0.89 normal；內臟脂肪10（1–10）剛入 normal。分段肌：臂2.0/2.0、軀幹18.2、腿6.1/6.1 全 normal 對稱。分段脂：臂1.6/1.6、軀幹11.1、腿3.3/3.3 均 High。唔採用理想53.9／控制−8.8／脂控−9.5。對 9/1 18:31 gym：體重−1.2、BFP−0.4pp、脂−0.7、肌−0.3、水−0.4、內臟11→10、Score69不變。9日移動含水分；唔當減咗0.7脂或跌肌。晏晝家秤62.55≠呢個62.7≠晨磅。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="64" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 morning</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 62.4。較9/9晨 62.95 −0.55（9/10無晨磅）。尋日日結690偏低＋gym＋43分斜路，腸空／肝醣水，同9/8 62.65（455後日）同一類。唔當減脂、唔當 dry、唔當新底。7日晨磅均約63.2（9/4–9/11，缺9/10晨：63.5／63.5／63.9／63.5／62.65／62.95／62.4）。晏晝家秤62.55同BIA 62.7唔當晨磅。今日仍≥~1200，唔好400–800。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 gym（完成）</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>無 gym room。Home 腹肌片 8min 後停（18min 片跟唔落）</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>Coffee 站立燃脂第一套完成。Apple Watch Mixed Cardio 18:54–19:29 San Tin；Workout 32:13／Elapsed 34:36；active 164／total 209 kcal；avg HR 128。用戶：比斜路辛苦。</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>完成。唔去gym。① 站立燃脂 34min 片跟完（錶 32:13，比斜路辛苦）。② 練腹片 https://youtu.be/7rp7DGEAJ-s 做 8min 停：好攰、太難、搞唔掂。手錶 164／209 唔扣食物。Total 唔當 TDEE。當心肺／核心日，唔當重量。唔加多套。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="64" customHeight="1">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12 morning</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>晨磅 62.2。較9/11晨 62.4 −0.2。連續62.x（9/8 62.65／9/9 62.95／9/11 62.4）後再低，當水／腸胃／肝醣，唔當減脂、唔當 dry、唔當新底。7日晨磅均約63.0（9/5–9/12，缺9/10晨：63.5／63.9／63.5／62.65／62.95／62.4／62.2）。晏晝家秤同BIA唔當晨磅。</t>
         </is>
       </c>
     </row>

</xml_diff>